<commit_message>
Planning 2-22/11 : règles journée de solidarité du 11/11, indispos Jennyfer 6/11 et Rose 7/11
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_2-22nov.xlsx
+++ b/Planning_2-22nov.xlsx
@@ -102,17 +102,17 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00A3A3A3"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00713F12"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00A3A3A3"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
@@ -149,7 +149,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -201,6 +201,11 @@
         <fgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDECC8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -228,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -268,10 +273,10 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -290,6 +295,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -799,25 +807,25 @@
 7h00</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>11:00 – 14:00
+15:00 – 19:00
+7h00</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>11:40 – 15:00
 16:00 – 19:40
 7h00</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
-        <is>
-          <t>11:00 – 14:00
-15:00 – 19:00
-7h00</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
           <t>11:40 – 15:00
@@ -825,7 +833,7 @@
 7h00</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
@@ -878,12 +886,12 @@
 7h00</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Indispo</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
@@ -913,26 +921,26 @@
 6h15</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>Indispo</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
@@ -957,27 +965,27 @@
 contrat 15h</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
@@ -1120,17 +1128,17 @@
 7h00</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F15" s="15" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>CP (solidarité)</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>11:00 – 14:00
 15:00 – 19:00
@@ -1180,31 +1188,31 @@
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
+          <t>10:00 – 14:00
+15:00 – 18:00
+7h00</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="inlineStr">
+        <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 17:50
 7h00</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="G16" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H16" s="16" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
@@ -1222,7 +1230,7 @@
 contrat 25h</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>Repos</t>
         </is>
@@ -1236,408 +1244,407 @@
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
+          <t>14:00 – 19:00
+5h00</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>23h45</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Sara
+contrat 15h</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>CP (solidarité)</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 18:30
+7h40</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>10:50 – 14:00
+15:00 – 19:10
+7h20</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>15h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Présents</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>3 pers.</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>3 pers.</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
+        <is>
+          <t>2 pers.</t>
+        </is>
+      </c>
+      <c r="I19" s="22" t="n"/>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>SEMAINE 3  ·  du lundi 16 novembre au dimanche 22 novembre</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Salarié</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Lun 16/11</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Mar 17/11</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Mer 18/11</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Jeu 19/11</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Ven 20/11</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Sam 21/11</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>Dim 22/11</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Yassine
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>11:00 – 14:00
+15:00 – 19:00
+7h00</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>11:40 – 15:00
+16:00 – 19:40
+7h00</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>35h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Rose
+contrat 35h</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>09:50 – 14:00
+15:00 – 17:50
+7h00</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>35h00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Jennyfer
+contrat 25h</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>12:25 – 15:00
 16:00 – 19:40
 6h15</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H17" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="I17" s="17" t="inlineStr">
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>12:25 – 15:00
+16:00 – 19:40
+6h15</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>12:25 – 15:00
+16:00 – 19:40
+6h15</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>11:55 – 15:00
+16:00 – 19:10
+6h15</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
         <is>
           <t>25h00</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="58" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Sara
 contrat 15h</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E18" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>09:50 – 14:00
 15:00 – 18:30
 7h40</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr">
+      <c r="H26" s="19" t="inlineStr">
         <is>
           <t>10:50 – 14:00
 15:00 – 19:10
 7h20</t>
         </is>
       </c>
-      <c r="I18" s="17" t="inlineStr">
-        <is>
-          <t>15h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>Présents</t>
-        </is>
-      </c>
-      <c r="B19" s="21" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="C19" s="21" t="inlineStr">
-        <is>
-          <t>3 pers.</t>
-        </is>
-      </c>
-      <c r="D19" s="21" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="E19" s="21" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr">
-        <is>
-          <t>3 pers.</t>
-        </is>
-      </c>
-      <c r="G19" s="21" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="H19" s="21" t="inlineStr">
-        <is>
-          <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="I19" s="22" t="n"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>SEMAINE 3  ·  du lundi 16 novembre au dimanche 22 novembre</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>Salarié</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Lun 16/11</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>Mar 17/11</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>Mer 18/11</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>Jeu 19/11</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>Ven 20/11</t>
-        </is>
-      </c>
-      <c r="G22" s="11" t="inlineStr">
-        <is>
-          <t>Sam 21/11</t>
-        </is>
-      </c>
-      <c r="H22" s="11" t="inlineStr">
-        <is>
-          <t>Dim 22/11</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Yassine
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B23" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>11:00 – 14:00
-15:00 – 19:00
-7h00</t>
-        </is>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>11:40 – 15:00
-16:00 – 19:40
-7h00</t>
-        </is>
-      </c>
-      <c r="H23" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="I23" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Rose
-contrat 35h</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="F24" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 17:50
-7h00</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H24" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="inlineStr">
-        <is>
-          <t>35h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="58" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Jennyfer
-contrat 25h</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>12:25 – 15:00
-16:00 – 19:40
-6h15</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="inlineStr">
-        <is>
-          <t>12:25 – 15:00
-16:00 – 19:40
-6h15</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>12:25 – 15:00
-16:00 – 19:40
-6h15</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="G25" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>11:55 – 15:00
-16:00 – 19:10
-6h15</t>
-        </is>
-      </c>
-      <c r="I25" s="17" t="inlineStr">
-        <is>
-          <t>25h00</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Sara
-contrat 15h</t>
-        </is>
-      </c>
-      <c r="B26" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="C26" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="E26" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="G26" s="14" t="inlineStr">
-        <is>
-          <t>09:50 – 14:00
-15:00 – 18:30
-7h40</t>
-        </is>
-      </c>
-      <c r="H26" s="19" t="inlineStr">
-        <is>
-          <t>10:50 – 14:00
-15:00 – 19:10
-7h20</t>
-        </is>
-      </c>
       <c r="I26" s="17" t="inlineStr">
         <is>
           <t>15h00</t>
@@ -1688,42 +1695,42 @@
       <c r="I27" s="22" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>À SAVOIR</t>
         </is>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
-      <c r="A30" s="24" t="inlineStr">
-        <is>
-          <t>• Rose toujours en ouverture (lun-ven, part à 17:50), Jennyfer toujours en fermeture, Yassine en fermeture ou milieu de journée ; le mardi Yassine est là dès 09:50 pour la commande (avant 11h).</t>
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>• Rose toujours en ouverture (lun-ven, part avant la fermeture), Jennyfer toujours en fermeture, Yassine en fermeture ou milieu de journée ; le mardi Yassine est là dès 09:50 pour la commande (avant 11h).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="24" t="inlineStr">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>• Dimanche à 2 : Sara + Jennyfer (8/11 et 22/11) ou Yassine (15/11). Sara ouvre le samedi et le dimanche.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="24" t="inlineStr">
-        <is>
-          <t>• Mercredi 11 novembre : journée de solidarité → magasin ouvert, Rose et Jennyfer travaillent normalement (journée non rémunérée en plus : 7h temps plein, au prorata pour les temps partiels).</t>
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>• Mer 11/11 journée de solidarité (mail CEDIF) : magasin ouvert 10:00-19:00 ; Rose 7h (maxi 35h = 7h), Jennyfer 5h (maxi 25h = 5h). Yassine et Sara sont en repos hebdomadaire ce jour-là → 1 jour de CP décompté (sauf s'ils préfèrent travailler, heures incluses dans leur semaine, sans heures supp).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>• Lundi 2 novembre : Jennyfer encore en congé.</t>
+      <c r="A33" s="25" t="inlineStr">
+        <is>
+          <t>• Indispos : Jennyfer en congé lun 2/11 et indispo ven 6/11 (Yassine ferme) · Rose indispo sam 7/11 (jour de repos de toute façon).</t>
         </is>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="25" t="inlineStr">
         <is>
           <t>• Livraisons : 3 personnes les jeu 5, ven 13 et jeu 19 ; 2 personnes les ven 6, jeu 12 et ven 20.</t>
         </is>

</xml_diff>

<commit_message>
11/11 : toute l'équipe en magasin sauf Sara, pas de CP solidarité
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sABE5Ku13TMCaT7NQhVkc
</commit_message>
<xml_diff>
--- a/Planning_2-22nov.xlsx
+++ b/Planning_2-22nov.xlsx
@@ -1128,21 +1128,21 @@
 7h00</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
-        <is>
-          <t>CP (solidarité)</t>
-        </is>
-      </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>Repos</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>11:00 – 14:00
 15:00 – 19:00
 7h00</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
@@ -1295,9 +1295,9 @@
           <t>Repos</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>CP (solidarité)</t>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Repos</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
@@ -1348,17 +1348,17 @@
       </c>
       <c r="D19" s="21" t="inlineStr">
         <is>
+          <t>3 pers.</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
           <t>2 pers.</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>2 pers.</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr">
-        <is>
-          <t>3 pers.</t>
         </is>
       </c>
       <c r="G19" s="21" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>• Mer 11/11 journée de solidarité (mail CEDIF) : magasin ouvert 10:00-19:00 ; Rose 7h (maxi 35h = 7h), Jennyfer 5h (maxi 25h = 5h). Yassine et Sara sont en repos hebdomadaire ce jour-là → 1 jour de CP décompté (sauf s'ils préfèrent travailler, heures incluses dans leur semaine, sans heures supp).</t>
+          <t>• Mer 11/11 journée de solidarité (mail CEDIF) : magasin ouvert 10:00-19:00 ; Rose 7h (maxi 35h = 7h), Jennyfer 5h (maxi 25h = 5h). Yassine 7h (inclus dans ses 35h : il ne vient pas le vendredi 13). Sara en repos. Pas de CP solidarité.</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="25" t="inlineStr">
         <is>
-          <t>• Livraisons : 3 personnes les jeu 5, ven 13 et jeu 19 ; 2 personnes les ven 6, jeu 12 et ven 20.</t>
+          <t>• Livraisons : 3 personnes les jeu 5 et jeu 19 ; 2 personnes les ven 6, jeu 12, ven 13 et ven 20.</t>
         </is>
       </c>
     </row>

</xml_diff>